<commit_message>
Added KM plots and viability contrasts
</commit_message>
<xml_diff>
--- a/data/SurvivalData.xlsx
+++ b/data/SurvivalData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Shared drives\Alphey Lab\Daisy Drive\Manuscripts\Cd fitness cost in An. stephensi\Clean_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ueanorwich-my.sharepoint.com/personal/hpd08ucu_uea_ac_uk/Documents/Manuscripts/cardinal_fitness/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2420DEB8-8887-476C-9145-B2383A2503A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{2420DEB8-8887-476C-9145-B2383A2503A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9136EC9A-C6C3-4FD3-AE53-4884C927869B}"/>
   <bookViews>
-    <workbookView xWindow="31455" yWindow="-3120" windowWidth="17640" windowHeight="16995" activeTab="1" xr2:uid="{51CB0BA6-2C65-423F-A414-15434B2754D4}"/>
+    <workbookView minimized="1" xWindow="31080" yWindow="2070" windowWidth="14400" windowHeight="8175" xr2:uid="{51CB0BA6-2C65-423F-A414-15434B2754D4}"/>
   </bookViews>
   <sheets>
     <sheet name="1759" sheetId="1" r:id="rId1"/>
@@ -571,7 +571,7 @@
         <v>12</v>
       </c>
       <c r="M3" s="1">
-        <f t="shared" ref="M2:N3" si="0">(E3+E5)/2</f>
+        <f t="shared" ref="M3:N3" si="0">(E3+E5)/2</f>
         <v>86.5</v>
       </c>
       <c r="N3" s="1">
@@ -852,6 +852,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C57D715A-D451-4EB5-A0D4-B781B4C2B161}">
   <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.08984375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">

</xml_diff>